<commit_message>
Repo hygiene: ignore logs/venv/tools, untrack watch_tamarac.log, sync data files
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings_Manual.xlsx
+++ b/data/Tamarac_Holdings_Manual.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5A2461E-E7D9-40B5-ACD9-863180BF669C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{E5A2461E-E7D9-40B5-ACD9-863180BF669C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFCDD470-657C-47B5-8553-DFBAC89F3311}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2B840D57-0EA2-494E-9DF5-3E4C4D0760AB}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2B840D57-0EA2-494E-9DF5-3E4C4D0760AB}"/>
   </bookViews>
   <sheets>
     <sheet name="QDVD" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,20 @@
     <sheet name="OR" sheetId="4" r:id="rId4"/>
     <sheet name="DCP" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -2326,17 +2339,16 @@
         <v>27327.39</v>
       </c>
       <c r="J32">
-        <v>0</v>
+        <v>3260</v>
       </c>
       <c r="K32" s="3">
         <v>9119.24</v>
       </c>
-      <c r="L32" t="str">
-        <f>""</f>
-        <v/>
+      <c r="L32" s="2">
+        <v>8.1299999999999997E-2</v>
       </c>
       <c r="M32" s="2">
-        <v>0</v>
+        <v>4.4699999999999997E-2</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
@@ -2647,7 +2659,7 @@
         <v>46132</v>
       </c>
       <c r="B2" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" ref="B2:B25" si="0">"*Quality SMID Dividend Strategy (*SMID)"</f>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C2" s="2">
@@ -2692,7 +2704,7 @@
         <v>46132</v>
       </c>
       <c r="B3" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C3" s="2">
@@ -2737,7 +2749,7 @@
         <v>46132</v>
       </c>
       <c r="B4" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C4" s="2">
@@ -2782,7 +2794,7 @@
         <v>46132</v>
       </c>
       <c r="B5" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C5" s="2">
@@ -2827,7 +2839,7 @@
         <v>46132</v>
       </c>
       <c r="B6" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C6" s="2">
@@ -2871,7 +2883,7 @@
         <v>46132</v>
       </c>
       <c r="B7" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C7" s="2">
@@ -2915,7 +2927,7 @@
         <v>46132</v>
       </c>
       <c r="B8" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C8" s="2">
@@ -2960,7 +2972,7 @@
         <v>46132</v>
       </c>
       <c r="B9" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C9" s="2">
@@ -3004,7 +3016,7 @@
         <v>46132</v>
       </c>
       <c r="B10" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C10" s="2">
@@ -3048,7 +3060,7 @@
         <v>46132</v>
       </c>
       <c r="B11" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C11" s="2">
@@ -3092,7 +3104,7 @@
         <v>46132</v>
       </c>
       <c r="B12" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C12" s="2">
@@ -3136,7 +3148,7 @@
         <v>46132</v>
       </c>
       <c r="B13" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C13" s="2">
@@ -3180,7 +3192,7 @@
         <v>46132</v>
       </c>
       <c r="B14" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C14" s="2">
@@ -3224,7 +3236,7 @@
         <v>46132</v>
       </c>
       <c r="B15" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C15" s="2">
@@ -3268,7 +3280,7 @@
         <v>46132</v>
       </c>
       <c r="B16" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C16" s="2">
@@ -3312,7 +3324,7 @@
         <v>46132</v>
       </c>
       <c r="B17" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C17" s="2">
@@ -3356,7 +3368,7 @@
         <v>46132</v>
       </c>
       <c r="B18" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C18" s="2">
@@ -3400,7 +3412,7 @@
         <v>46132</v>
       </c>
       <c r="B19" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C19" s="2">
@@ -3445,7 +3457,7 @@
         <v>46132</v>
       </c>
       <c r="B20" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C20" s="2">
@@ -3490,7 +3502,7 @@
         <v>46132</v>
       </c>
       <c r="B21" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C21" s="2">
@@ -3534,7 +3546,7 @@
         <v>46132</v>
       </c>
       <c r="B22" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C22" s="2">
@@ -3578,7 +3590,7 @@
         <v>46132</v>
       </c>
       <c r="B23" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C23" s="2">
@@ -3622,7 +3634,7 @@
         <v>46132</v>
       </c>
       <c r="B24" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C24" s="2">
@@ -3667,7 +3679,7 @@
         <v>46132</v>
       </c>
       <c r="B25" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C25" s="2">
@@ -3793,7 +3805,7 @@
         <v>46132</v>
       </c>
       <c r="B2" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" ref="B2:B47" si="0">"*Quality All-Cap Dividend Strategy (*DAC)"</f>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C2" s="2">
@@ -3838,7 +3850,7 @@
         <v>46132</v>
       </c>
       <c r="B3" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C3" s="2">
@@ -3883,7 +3895,7 @@
         <v>46132</v>
       </c>
       <c r="B4" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C4" s="2">
@@ -3928,7 +3940,7 @@
         <v>46132</v>
       </c>
       <c r="B5" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C5" s="2">
@@ -3973,7 +3985,7 @@
         <v>46132</v>
       </c>
       <c r="B6" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C6" s="2">
@@ -4018,7 +4030,7 @@
         <v>46132</v>
       </c>
       <c r="B7" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C7" s="2">
@@ -4062,7 +4074,7 @@
         <v>46132</v>
       </c>
       <c r="B8" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C8" s="2">
@@ -4107,7 +4119,7 @@
         <v>46132</v>
       </c>
       <c r="B9" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C9" s="2">
@@ -4151,7 +4163,7 @@
         <v>46132</v>
       </c>
       <c r="B10" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C10" s="2">
@@ -4196,7 +4208,7 @@
         <v>46132</v>
       </c>
       <c r="B11" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C11" s="2">
@@ -4240,7 +4252,7 @@
         <v>46132</v>
       </c>
       <c r="B12" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C12" s="2">
@@ -4285,7 +4297,7 @@
         <v>46132</v>
       </c>
       <c r="B13" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C13" s="2">
@@ -4329,7 +4341,7 @@
         <v>46132</v>
       </c>
       <c r="B14" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C14" s="2">
@@ -4374,7 +4386,7 @@
         <v>46132</v>
       </c>
       <c r="B15" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C15" s="2">
@@ -4419,7 +4431,7 @@
         <v>46132</v>
       </c>
       <c r="B16" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C16" s="2">
@@ -4463,7 +4475,7 @@
         <v>46132</v>
       </c>
       <c r="B17" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C17" s="2">
@@ -4507,7 +4519,7 @@
         <v>46132</v>
       </c>
       <c r="B18" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C18" s="2">
@@ -4551,7 +4563,7 @@
         <v>46132</v>
       </c>
       <c r="B19" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C19" s="2">
@@ -4595,7 +4607,7 @@
         <v>46132</v>
       </c>
       <c r="B20" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C20" s="2">
@@ -4639,7 +4651,7 @@
         <v>46132</v>
       </c>
       <c r="B21" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C21" s="2">
@@ -4683,7 +4695,7 @@
         <v>46132</v>
       </c>
       <c r="B22" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C22" s="2">
@@ -4727,7 +4739,7 @@
         <v>46132</v>
       </c>
       <c r="B23" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C23" s="2">
@@ -4772,7 +4784,7 @@
         <v>46132</v>
       </c>
       <c r="B24" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C24" s="2">
@@ -4816,7 +4828,7 @@
         <v>46132</v>
       </c>
       <c r="B25" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C25" s="2">
@@ -4860,7 +4872,7 @@
         <v>46132</v>
       </c>
       <c r="B26" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C26" s="2">
@@ -4905,7 +4917,7 @@
         <v>46132</v>
       </c>
       <c r="B27" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C27" s="2">
@@ -4949,7 +4961,7 @@
         <v>46132</v>
       </c>
       <c r="B28" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C28" s="2">
@@ -4993,7 +5005,7 @@
         <v>46132</v>
       </c>
       <c r="B29" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C29" s="2">
@@ -5037,7 +5049,7 @@
         <v>46132</v>
       </c>
       <c r="B30" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C30" s="2">
@@ -5081,7 +5093,7 @@
         <v>46132</v>
       </c>
       <c r="B31" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C31" s="2">
@@ -5125,7 +5137,7 @@
         <v>46132</v>
       </c>
       <c r="B32" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C32" s="2">
@@ -5169,7 +5181,7 @@
         <v>46132</v>
       </c>
       <c r="B33" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C33" s="2">
@@ -5213,7 +5225,7 @@
         <v>46132</v>
       </c>
       <c r="B34" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C34" s="2">
@@ -5257,7 +5269,7 @@
         <v>46132</v>
       </c>
       <c r="B35" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C35" s="2">
@@ -5302,7 +5314,7 @@
         <v>46132</v>
       </c>
       <c r="B36" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C36" s="2">
@@ -5346,7 +5358,7 @@
         <v>46132</v>
       </c>
       <c r="B37" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C37" s="2">
@@ -5391,7 +5403,7 @@
         <v>46132</v>
       </c>
       <c r="B38" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C38" s="2">
@@ -5435,7 +5447,7 @@
         <v>46132</v>
       </c>
       <c r="B39" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C39" s="2">
@@ -5479,7 +5491,7 @@
         <v>46132</v>
       </c>
       <c r="B40" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C40" s="2">
@@ -5523,7 +5535,7 @@
         <v>46132</v>
       </c>
       <c r="B41" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C41" s="2">
@@ -5567,7 +5579,7 @@
         <v>46132</v>
       </c>
       <c r="B42" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C42" s="2">
@@ -5612,7 +5624,7 @@
         <v>46132</v>
       </c>
       <c r="B43" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C43" s="2">
@@ -5656,7 +5668,7 @@
         <v>46132</v>
       </c>
       <c r="B44" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C44" s="2">
@@ -5700,7 +5712,7 @@
         <v>46132</v>
       </c>
       <c r="B45" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C45" s="2">
@@ -5744,7 +5756,7 @@
         <v>46132</v>
       </c>
       <c r="B46" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C46" s="2">
@@ -5789,7 +5801,7 @@
         <v>46132</v>
       </c>
       <c r="B47" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C47" s="2">
@@ -5915,7 +5927,7 @@
         <v>46132</v>
       </c>
       <c r="B2" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" ref="B2:B36" si="0">"*Oregon Dividend Strategy (*QDGR)"</f>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C2" s="2">
@@ -5960,7 +5972,7 @@
         <v>46132</v>
       </c>
       <c r="B3" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C3" s="2">
@@ -6005,7 +6017,7 @@
         <v>46132</v>
       </c>
       <c r="B4" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C4" s="2">
@@ -6050,7 +6062,7 @@
         <v>46132</v>
       </c>
       <c r="B5" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C5" s="2">
@@ -6094,7 +6106,7 @@
         <v>46132</v>
       </c>
       <c r="B6" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C6" s="2">
@@ -6139,7 +6151,7 @@
         <v>46132</v>
       </c>
       <c r="B7" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C7" s="2">
@@ -6183,7 +6195,7 @@
         <v>46132</v>
       </c>
       <c r="B8" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C8" s="2">
@@ -6227,7 +6239,7 @@
         <v>46132</v>
       </c>
       <c r="B9" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C9" s="2">
@@ -6272,7 +6284,7 @@
         <v>46132</v>
       </c>
       <c r="B10" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C10" s="2">
@@ -6316,7 +6328,7 @@
         <v>46132</v>
       </c>
       <c r="B11" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C11" s="2">
@@ -6360,7 +6372,7 @@
         <v>46132</v>
       </c>
       <c r="B12" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C12" s="2">
@@ -6404,7 +6416,7 @@
         <v>46132</v>
       </c>
       <c r="B13" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C13" s="2">
@@ -6448,7 +6460,7 @@
         <v>46132</v>
       </c>
       <c r="B14" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C14" s="2">
@@ -6493,7 +6505,7 @@
         <v>46132</v>
       </c>
       <c r="B15" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C15" s="2">
@@ -6537,7 +6549,7 @@
         <v>46132</v>
       </c>
       <c r="B16" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C16" s="2">
@@ -6581,7 +6593,7 @@
         <v>46132</v>
       </c>
       <c r="B17" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C17" s="2">
@@ -6626,7 +6638,7 @@
         <v>46132</v>
       </c>
       <c r="B18" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C18" s="2">
@@ -6670,7 +6682,7 @@
         <v>46132</v>
       </c>
       <c r="B19" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C19" s="2">
@@ -6714,7 +6726,7 @@
         <v>46132</v>
       </c>
       <c r="B20" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C20" s="2">
@@ -6758,7 +6770,7 @@
         <v>46132</v>
       </c>
       <c r="B21" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C21" s="2">
@@ -6802,7 +6814,7 @@
         <v>46132</v>
       </c>
       <c r="B22" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C22" s="2">
@@ -6846,7 +6858,7 @@
         <v>46132</v>
       </c>
       <c r="B23" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C23" s="2">
@@ -6890,7 +6902,7 @@
         <v>46132</v>
       </c>
       <c r="B24" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C24" s="2">
@@ -6934,7 +6946,7 @@
         <v>46132</v>
       </c>
       <c r="B25" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C25" s="2">
@@ -6979,7 +6991,7 @@
         <v>46132</v>
       </c>
       <c r="B26" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C26" s="2">
@@ -7023,7 +7035,7 @@
         <v>46132</v>
       </c>
       <c r="B27" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C27" s="2">
@@ -7068,7 +7080,7 @@
         <v>46132</v>
       </c>
       <c r="B28" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C28" s="2">
@@ -7112,7 +7124,7 @@
         <v>46132</v>
       </c>
       <c r="B29" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C29" s="2">
@@ -7156,7 +7168,7 @@
         <v>46132</v>
       </c>
       <c r="B30" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C30" s="2">
@@ -7201,7 +7213,7 @@
         <v>46132</v>
       </c>
       <c r="B31" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C31" s="2">
@@ -7245,7 +7257,7 @@
         <v>46132</v>
       </c>
       <c r="B32" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C32" s="2">
@@ -7289,7 +7301,7 @@
         <v>46132</v>
       </c>
       <c r="B33" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C33" s="2">
@@ -7333,7 +7345,7 @@
         <v>46132</v>
       </c>
       <c r="B34" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C34" s="2">
@@ -7377,7 +7389,7 @@
         <v>46132</v>
       </c>
       <c r="B35" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C35" s="2">
@@ -7422,7 +7434,7 @@
         <v>46132</v>
       </c>
       <c r="B36" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C36" s="2">
@@ -9466,6 +9478,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
     <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
@@ -9678,15 +9699,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -9702,13 +9714,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0AD8D72A-0055-48C6-BD08-3D90393D055A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA66E9F4-50C0-4090-B730-CDDB44A38EC9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA66E9F4-50C0-4090-B730-CDDB44A38EC9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0AD8D72A-0055-48C6-BD08-3D90393D055A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB7A8652-D143-4B7B-96CD-BAC47B743C9D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB7A8652-D143-4B7B-96CD-BAC47B743C9D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Tamarac manual file (Tamarac_Holdings_Manual.xlsx) 2026-06-03 09:26
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings_Manual.xlsx
+++ b/data/Tamarac_Holdings_Manual.xlsx
@@ -12844,4 +12844,252 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CEF7208-21A5-4BAE-AE89-10F9C7FEA31D}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD098924-8D31-400A-A91F-FD68F8836EA6}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC1A2E93-697F-48B6-9CBA-2967B661829E}"/>
 </file>
</xml_diff>